<commit_message>
last fix before move to production
</commit_message>
<xml_diff>
--- a/docs/DB詳細設計.xlsx
+++ b/docs/DB詳細設計.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos2\selfdrinkbar-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D036FA-7AB8-445F-B79F-2D97DF635CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA3DB46-0083-49BA-BEF7-704B19DB08D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{6E515E34-1608-4F1D-8466-1D4D7610F251}"/>
+    <workbookView xWindow="-28590" yWindow="360" windowWidth="28485" windowHeight="14595" activeTab="3" xr2:uid="{6E515E34-1608-4F1D-8466-1D4D7610F251}"/>
   </bookViews>
   <sheets>
     <sheet name="DB定義書_orders" sheetId="1" r:id="rId1"/>
-    <sheet name="DB定義書_ordered_item" sheetId="2" r:id="rId2"/>
+    <sheet name="DB定義書_order_details" sheetId="2" r:id="rId2"/>
     <sheet name="DB定義書_items" sheetId="3" r:id="rId3"/>
     <sheet name="DB定義書_admins" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="115">
   <si>
     <t>カラム名</t>
   </si>
@@ -125,9 +125,6 @@
     <t>VARCHAR(255)</t>
   </si>
   <si>
-    <t>VARCHAR(20)</t>
-  </si>
-  <si>
     <t>■ リレーション</t>
   </si>
   <si>
@@ -140,9 +137,6 @@
     <t>1 対 多</t>
   </si>
   <si>
-    <t>■ ステータス仕様（membership_status）</t>
-  </si>
-  <si>
     <t>値</t>
   </si>
   <si>
@@ -159,9 +153,6 @@
     <t>備考</t>
   </si>
   <si>
-    <t>role により権限を制御（admin / super）</t>
-  </si>
-  <si>
     <t>管理者ID（PK, AUTO_INCREMENT）</t>
   </si>
   <si>
@@ -175,14 +166,6 @@
   </si>
   <si>
     <t>4. admins テーブル（管理者情報）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者（user）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>上位管理者（super）</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -449,15 +432,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>about</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>created_at</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>status</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -486,51 +461,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>販売中/非表示のどちらか</t>
-    <rPh sb="0" eb="3">
-      <t>ハンバイチュウ</t>
-    </rPh>
-    <rPh sb="4" eb="7">
-      <t>ヒヒョウジ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>販売中</t>
-    <rPh sb="0" eb="3">
-      <t>ハンバイチュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>非表示（販売停止）</t>
-    <rPh sb="0" eb="3">
-      <t>ヒヒョウジ</t>
-    </rPh>
-    <rPh sb="4" eb="8">
-      <t>ハンバイテイシ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>権限（管理者 / 上位管理者）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>上位管理者</t>
-    <rPh sb="0" eb="5">
-      <t>ジョウイカンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>親注文ID</t>
     <rPh sb="0" eb="1">
       <t>オヤ</t>
@@ -555,10 +485,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>FK→items.id</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>購入時の商品名（履歴用）</t>
     <rPh sb="0" eb="3">
       <t>コウニュウジ</t>
@@ -621,18 +547,81 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>items.id → ordered_items.item_id</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>非表示</t>
-    <rPh sb="0" eb="3">
-      <t>ヒヒョウジ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>UK</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デモ用管理者（demo）</t>
+    <rPh sb="2" eb="3">
+      <t>ヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>通常管理者（admin）</t>
+    <rPh sb="0" eb="2">
+      <t>ツウジョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>demo</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>role により権限を制御（demo / admin）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>description</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>タイムスタンプ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>category</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VARCHAR(50)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商品カテゴリー</t>
+    <rPh sb="0" eb="2">
+      <t>ショウヒン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ｄ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>updated_at</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>更新日時</t>
+    <rPh sb="0" eb="2">
+      <t>コウシン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ニチジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>権限（デモ管理者 / 通常管理者）</t>
+    <rPh sb="11" eb="13">
+      <t>ツウジョウ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1054,7 +1043,7 @@
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="2:6" x14ac:dyDescent="0.4">
@@ -1075,7 +1064,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.4">
@@ -1083,7 +1072,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.4">
@@ -1127,15 +1116,15 @@
         <v>5</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B11" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>4</v>
@@ -1147,12 +1136,12 @@
         <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>10</v>
@@ -1164,15 +1153,15 @@
         <v>25</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B13" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>5</v>
@@ -1181,20 +1170,20 @@
         <v>25</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>2</v>
@@ -1202,50 +1191,50 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B17" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B19" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B20" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B21" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B22" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B23" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1256,7 +1245,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A6CF-D514-4BB7-B848-34EDD9B7D9A7}">
-  <dimension ref="B1:F24"/>
+  <dimension ref="B1:F25"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="4.375" bestFit="1" customWidth="1"/>
@@ -1272,7 +1261,7 @@
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="2:6" x14ac:dyDescent="0.4">
@@ -1293,7 +1282,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.4">
@@ -1301,7 +1290,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.4">
@@ -1314,10 +1303,10 @@
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B7" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.4">
@@ -1353,15 +1342,15 @@
         <v>5</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B12" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>4</v>
@@ -1370,15 +1359,15 @@
         <v>5</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B13" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>4</v>
@@ -1387,18 +1376,18 @@
         <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
@@ -1407,12 +1396,12 @@
         <v>25</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B15" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>4</v>
@@ -1424,12 +1413,12 @@
         <v>25</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B16" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>4</v>
@@ -1441,15 +1430,15 @@
         <v>25</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B17" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>5</v>
@@ -1458,48 +1447,65 @@
         <v>25</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.4">
-      <c r="B20" t="s">
-        <v>28</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B18" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.4">
-      <c r="B21" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>2</v>
+      <c r="B21" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B22" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>109</v>
+        <v>29</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>110</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B23" s="1" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" s="2" customFormat="1" x14ac:dyDescent="0.4"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B24" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" s="2" customFormat="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1508,7 +1514,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5461AF-EFF5-4885-8B93-D951903C8A7C}">
-  <dimension ref="B1:F25"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="4.375" bestFit="1" customWidth="1"/>
@@ -1522,17 +1528,17 @@
     <col min="9" max="9" width="19.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
@@ -1540,23 +1546,23 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B4" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.4">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B6" s="1" t="s">
         <v>21</v>
       </c>
@@ -1564,12 +1570,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
@@ -1586,7 +1592,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1597,18 +1603,18 @@
         <v>5</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>5</v>
@@ -1617,29 +1623,29 @@
         <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B12" s="1" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>111</v>
+        <v>5</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>25</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.4">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B13" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>4</v>
@@ -1651,32 +1657,35 @@
         <v>25</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.4">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B14" s="1" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>25</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.4">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>111</v>
+      </c>
       <c r="B15" s="1" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>5</v>
@@ -1685,63 +1694,24 @@
         <v>25</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B19" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B22" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B23" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B24" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B25" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1768,12 +1738,12 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.4">
@@ -1797,7 +1767,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.4">
@@ -1810,10 +1780,10 @@
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B8" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.4">
@@ -1849,15 +1819,15 @@
         <v>5</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B13" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>26</v>
@@ -1866,10 +1836,10 @@
         <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.4">
@@ -1877,7 +1847,7 @@
         <v>14</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
@@ -1886,7 +1856,7 @@
         <v>25</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.4">
@@ -1942,31 +1912,31 @@
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B19" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B20" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B21" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B22" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>